<commit_message>
chore: update 5 files
</commit_message>
<xml_diff>
--- a/public/word_upload_template.xlsx
+++ b/public/word_upload_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t xml:space="preserve">english_word</t>
   </si>
@@ -49,6 +49,9 @@
     <t xml:space="preserve">antonyms</t>
   </si>
   <si>
+    <t xml:space="preserve">Example-word</t>
+  </si>
+  <si>
     <t xml:space="preserve">exmple-word</t>
   </si>
   <si>
@@ -71,6 +74,9 @@
   </si>
   <si>
     <t xml:space="preserve">less, not regular, many</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example-word2</t>
   </si>
   <si>
     <t xml:space="preserve">Exmple-word2</t>
@@ -399,57 +405,57 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update 2 files
</commit_message>
<xml_diff>
--- a/public/word_upload_template.xlsx
+++ b/public/word_upload_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t xml:space="preserve">english_word</t>
   </si>
@@ -74,21 +74,6 @@
   </si>
   <si>
     <t xml:space="preserve">less, not regular, many</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example-word2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exmple-word2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exmple-word meaning2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">some2, many2, regular2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">less2, not regular2, many2</t>
   </si>
 </sst>
 </file>
@@ -368,7 +353,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="22.21875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -429,35 +414,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>22</v>
-      </c>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
chore: update 9 files
</commit_message>
<xml_diff>
--- a/public/word_upload_template.xlsx
+++ b/public/word_upload_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t xml:space="preserve">english_word</t>
   </si>
@@ -31,12 +31,12 @@
     <t xml:space="preserve">english_meaning</t>
   </si>
   <si>
+    <t xml:space="preserve">phonetics</t>
+  </si>
+  <si>
     <t xml:space="preserve">part_of_speech</t>
   </si>
   <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
     <t xml:space="preserve">class</t>
   </si>
   <si>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">antonyms</t>
   </si>
   <si>
-    <t xml:space="preserve">Example-word</t>
+    <t xml:space="preserve">Example-word-2</t>
   </si>
   <si>
     <t xml:space="preserve">exmple-word</t>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t xml:space="preserve">noun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test</t>
   </si>
   <si>
     <t xml:space="preserve">Pre-Primary1, class 1</t>
@@ -83,7 +80,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,12 +102,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -160,7 +151,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -353,40 +344,40 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="22.21875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -395,26 +386,25 @@
       <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="0" t="s">
-        <v>17</v>
-      </c>
     </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>